<commit_message>
style: add 5 more rows for item list and rendered the PR code in PDF
</commit_message>
<xml_diff>
--- a/procurement_documents/Purchase Request Excel Template (2).xlsx
+++ b/procurement_documents/Purchase Request Excel Template (2).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{990F3B20-0CDE-4616-BB10-DFCDB808DC9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DFC5EEB-505F-4BF0-99E5-5B6A669C4339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="947" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="CHEM_1" sheetId="59" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">CHEM_1!$A$1:$G$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">CHEM_1!$A$1:$G$53</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -807,7 +807,7 @@
     </xf>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -879,12 +879,6 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="2" borderId="0" xfId="9" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -897,199 +891,147 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="39" fontId="25" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="39" fontId="25" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="22" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="36" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="18" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="39" fontId="25" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="25" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1097,9 +1039,37 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="22" fontId="21" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma" xfId="9" builtinId="3"/>
@@ -1641,7 +1611,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:N53"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.28515625" style="3" customWidth="1"/>
@@ -1668,62 +1638,62 @@
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14"/>
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="105" t="s">
+      <c r="C2" s="40"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="56"/>
-      <c r="G2" s="35"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="41"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15"/>
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="57"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="101" t="s">
+      <c r="C3" s="42"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="F3" s="99"/>
-      <c r="G3" s="102" t="s">
+      <c r="F3" s="36"/>
+      <c r="G3" s="39" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14"/>
-      <c r="B4" s="56"/>
-      <c r="C4" s="56"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="99"/>
-      <c r="F4" s="99"/>
-      <c r="G4" s="100"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="37"/>
     </row>
     <row r="5" spans="1:14" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="58"/>
-      <c r="B5" s="59" t="s">
+      <c r="A5" s="31"/>
+      <c r="B5" s="81" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="59"/>
-      <c r="D5" s="63"/>
-      <c r="E5" s="103" t="s">
+      <c r="C5" s="81"/>
+      <c r="D5" s="82"/>
+      <c r="E5" s="83" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="103"/>
-      <c r="G5" s="104"/>
+      <c r="F5" s="83"/>
+      <c r="G5" s="84"/>
     </row>
     <row r="6" spans="1:14" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="60"/>
-      <c r="B6" s="61"/>
-      <c r="C6" s="61"/>
-      <c r="D6" s="61"/>
-      <c r="E6" s="61"/>
-      <c r="F6" s="61"/>
-      <c r="G6" s="61"/>
+      <c r="A6" s="16"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
     </row>
     <row r="7" spans="1:14" ht="21.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="16"/>
@@ -1735,40 +1705,40 @@
       <c r="G7" s="17"/>
     </row>
     <row r="8" spans="1:14" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="69"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="30" t="s">
+      <c r="B8" s="85"/>
+      <c r="C8" s="86"/>
+      <c r="D8" s="87"/>
+      <c r="E8" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="68"/>
-      <c r="G8" s="39"/>
+      <c r="F8" s="88"/>
+      <c r="G8" s="89"/>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:14" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="31" t="s">
+      <c r="A9" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="67"/>
-      <c r="C9" s="40"/>
-      <c r="D9" s="41"/>
-      <c r="E9" s="32" t="s">
+      <c r="B9" s="90"/>
+      <c r="C9" s="91"/>
+      <c r="D9" s="92"/>
+      <c r="E9" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="65"/>
-      <c r="G9" s="66"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="94"/>
     </row>
     <row r="10" spans="1:14" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="64"/>
-      <c r="B10" s="64"/>
-      <c r="C10" s="64"/>
-      <c r="D10" s="64"/>
-      <c r="E10" s="64"/>
-      <c r="F10" s="64"/>
-      <c r="G10" s="64"/>
+      <c r="A10" s="95"/>
+      <c r="B10" s="95"/>
+      <c r="C10" s="95"/>
+      <c r="D10" s="95"/>
+      <c r="E10" s="95"/>
+      <c r="F10" s="95"/>
+      <c r="G10" s="95"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
@@ -1777,14 +1747,14 @@
       <c r="B11" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C11" s="42" t="s">
+      <c r="C11" s="77" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="43"/>
-      <c r="E11" s="42" t="s">
+      <c r="D11" s="78"/>
+      <c r="E11" s="77" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="43"/>
+      <c r="F11" s="78"/>
       <c r="G11" s="22" t="s">
         <v>4</v>
       </c>
@@ -1792,10 +1762,10 @@
     <row r="12" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="12"/>
       <c r="B12" s="1"/>
-      <c r="C12" s="36"/>
-      <c r="D12" s="70"/>
-      <c r="E12" s="49"/>
-      <c r="F12" s="50"/>
+      <c r="C12" s="75"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="69"/>
+      <c r="F12" s="70"/>
       <c r="G12" s="23"/>
       <c r="H12" s="11"/>
       <c r="I12" s="5"/>
@@ -1808,10 +1778,10 @@
     <row r="13" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="12"/>
       <c r="B13" s="1"/>
-      <c r="C13" s="36"/>
-      <c r="D13" s="70"/>
-      <c r="E13" s="49"/>
-      <c r="F13" s="50"/>
+      <c r="C13" s="75"/>
+      <c r="D13" s="76"/>
+      <c r="E13" s="69"/>
+      <c r="F13" s="70"/>
       <c r="G13" s="23"/>
       <c r="H13" s="11"/>
       <c r="I13" s="8"/>
@@ -1822,401 +1792,461 @@
     <row r="14" spans="1:14" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="70"/>
-      <c r="E14" s="49"/>
-      <c r="F14" s="50"/>
+      <c r="C14" s="75"/>
+      <c r="D14" s="76"/>
+      <c r="E14" s="69"/>
+      <c r="F14" s="70"/>
       <c r="G14" s="23"/>
       <c r="H14" s="11"/>
     </row>
     <row r="15" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="70"/>
-      <c r="E15" s="49"/>
-      <c r="F15" s="50"/>
+      <c r="C15" s="75"/>
+      <c r="D15" s="76"/>
+      <c r="E15" s="69"/>
+      <c r="F15" s="70"/>
       <c r="G15" s="23"/>
       <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13"/>
       <c r="B16" s="2"/>
-      <c r="C16" s="36"/>
-      <c r="D16" s="70"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="50"/>
+      <c r="C16" s="75"/>
+      <c r="D16" s="76"/>
+      <c r="E16" s="69"/>
+      <c r="F16" s="70"/>
       <c r="G16" s="23"/>
       <c r="H16" s="11"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13"/>
       <c r="B17" s="2"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="70"/>
-      <c r="E17" s="49"/>
-      <c r="F17" s="50"/>
+      <c r="C17" s="75"/>
+      <c r="D17" s="76"/>
+      <c r="E17" s="69"/>
+      <c r="F17" s="70"/>
       <c r="G17" s="23"/>
       <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13"/>
       <c r="B18" s="2"/>
-      <c r="C18" s="44"/>
-      <c r="D18" s="71"/>
-      <c r="E18" s="49"/>
-      <c r="F18" s="50"/>
+      <c r="C18" s="71"/>
+      <c r="D18" s="72"/>
+      <c r="E18" s="69"/>
+      <c r="F18" s="70"/>
       <c r="G18" s="23"/>
       <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="13"/>
       <c r="B19" s="2"/>
-      <c r="C19" s="44"/>
-      <c r="D19" s="71"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="50"/>
+      <c r="C19" s="71"/>
+      <c r="D19" s="72"/>
+      <c r="E19" s="69"/>
+      <c r="F19" s="70"/>
       <c r="G19" s="23"/>
       <c r="H19" s="10"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13"/>
       <c r="B20" s="2"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="71"/>
-      <c r="E20" s="49"/>
-      <c r="F20" s="50"/>
+      <c r="C20" s="71"/>
+      <c r="D20" s="72"/>
+      <c r="E20" s="69"/>
+      <c r="F20" s="70"/>
       <c r="G20" s="23"/>
       <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="13"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="71"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="50"/>
+      <c r="C21" s="71"/>
+      <c r="D21" s="72"/>
+      <c r="E21" s="69"/>
+      <c r="F21" s="70"/>
       <c r="G21" s="23"/>
       <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="13"/>
       <c r="B22" s="2"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="71"/>
-      <c r="E22" s="49"/>
-      <c r="F22" s="50"/>
+      <c r="C22" s="71"/>
+      <c r="D22" s="72"/>
+      <c r="E22" s="69"/>
+      <c r="F22" s="70"/>
       <c r="G22" s="23"/>
       <c r="H22" s="10"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="44"/>
-      <c r="D23" s="71"/>
-      <c r="E23" s="49"/>
-      <c r="F23" s="50"/>
+      <c r="C23" s="71"/>
+      <c r="D23" s="72"/>
+      <c r="E23" s="69"/>
+      <c r="F23" s="70"/>
       <c r="G23" s="23"/>
       <c r="H23" s="10"/>
     </row>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="13"/>
       <c r="B24" s="2"/>
-      <c r="C24" s="44"/>
-      <c r="D24" s="71"/>
-      <c r="E24" s="49"/>
-      <c r="F24" s="50"/>
+      <c r="C24" s="71"/>
+      <c r="D24" s="72"/>
+      <c r="E24" s="69"/>
+      <c r="F24" s="70"/>
       <c r="G24" s="23"/>
       <c r="H24" s="10"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="13"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="44"/>
-      <c r="D25" s="71"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="50"/>
+      <c r="C25" s="71"/>
+      <c r="D25" s="72"/>
+      <c r="E25" s="69"/>
+      <c r="F25" s="70"/>
       <c r="G25" s="23"/>
       <c r="H25" s="10"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="13"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="44"/>
-      <c r="D26" s="71"/>
-      <c r="E26" s="49"/>
-      <c r="F26" s="50"/>
+      <c r="C26" s="71"/>
+      <c r="D26" s="72"/>
+      <c r="E26" s="69"/>
+      <c r="F26" s="70"/>
       <c r="G26" s="23"/>
       <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="13"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="44"/>
-      <c r="D27" s="71"/>
-      <c r="E27" s="49"/>
-      <c r="F27" s="50"/>
+      <c r="C27" s="71"/>
+      <c r="D27" s="72"/>
+      <c r="E27" s="69"/>
+      <c r="F27" s="70"/>
       <c r="G27" s="23"/>
       <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="13"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="45"/>
-      <c r="D28" s="46"/>
-      <c r="E28" s="49"/>
-      <c r="F28" s="50"/>
+      <c r="C28" s="73"/>
+      <c r="D28" s="74"/>
+      <c r="E28" s="69"/>
+      <c r="F28" s="70"/>
       <c r="G28" s="23"/>
       <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="13"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="45"/>
-      <c r="D29" s="46"/>
-      <c r="E29" s="49"/>
-      <c r="F29" s="50"/>
+      <c r="C29" s="73"/>
+      <c r="D29" s="74"/>
+      <c r="E29" s="69"/>
+      <c r="F29" s="70"/>
       <c r="G29" s="23"/>
       <c r="H29" s="10"/>
     </row>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="13"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="45"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="49"/>
-      <c r="F30" s="50"/>
+      <c r="C30" s="73"/>
+      <c r="D30" s="74"/>
+      <c r="E30" s="69"/>
+      <c r="F30" s="70"/>
       <c r="G30" s="23"/>
       <c r="H30" s="10"/>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="13"/>
       <c r="B31" s="2"/>
-      <c r="C31" s="44"/>
-      <c r="D31" s="71"/>
-      <c r="E31" s="49"/>
-      <c r="F31" s="50"/>
+      <c r="C31" s="71"/>
+      <c r="D31" s="72"/>
+      <c r="E31" s="69"/>
+      <c r="F31" s="70"/>
       <c r="G31" s="23"/>
       <c r="H31" s="10"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="13"/>
       <c r="B32" s="2"/>
-      <c r="C32" s="44"/>
-      <c r="D32" s="71"/>
-      <c r="E32" s="49"/>
-      <c r="F32" s="50"/>
+      <c r="C32" s="71"/>
+      <c r="D32" s="72"/>
+      <c r="E32" s="69"/>
+      <c r="F32" s="70"/>
       <c r="G32" s="23"/>
       <c r="H32" s="10"/>
     </row>
     <row r="33" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13"/>
       <c r="B33" s="2"/>
-      <c r="C33" s="44"/>
-      <c r="D33" s="71"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="50"/>
+      <c r="C33" s="71"/>
+      <c r="D33" s="72"/>
+      <c r="E33" s="69"/>
+      <c r="F33" s="70"/>
       <c r="G33" s="23"/>
       <c r="H33" s="10"/>
     </row>
     <row r="34" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13"/>
       <c r="B34" s="2"/>
-      <c r="C34" s="44"/>
-      <c r="D34" s="71"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="50"/>
+      <c r="C34" s="71"/>
+      <c r="D34" s="72"/>
+      <c r="E34" s="69"/>
+      <c r="F34" s="70"/>
       <c r="G34" s="23"/>
       <c r="H34" s="10"/>
     </row>
     <row r="35" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="13"/>
       <c r="B35" s="2"/>
-      <c r="C35" s="44"/>
-      <c r="D35" s="71"/>
-      <c r="E35" s="49"/>
-      <c r="F35" s="50"/>
+      <c r="C35" s="71"/>
+      <c r="D35" s="72"/>
+      <c r="E35" s="69"/>
+      <c r="F35" s="70"/>
       <c r="G35" s="23"/>
       <c r="H35" s="10"/>
     </row>
     <row r="36" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="13"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="44"/>
-      <c r="D36" s="71"/>
-      <c r="E36" s="49"/>
-      <c r="F36" s="50"/>
+      <c r="C36" s="71"/>
+      <c r="D36" s="72"/>
+      <c r="E36" s="69"/>
+      <c r="F36" s="70"/>
       <c r="G36" s="23"/>
       <c r="H36" s="10"/>
     </row>
     <row r="37" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="13"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="44"/>
-      <c r="D37" s="71"/>
-      <c r="E37" s="49"/>
-      <c r="F37" s="50"/>
+      <c r="C37" s="71"/>
+      <c r="D37" s="72"/>
+      <c r="E37" s="69"/>
+      <c r="F37" s="70"/>
       <c r="G37" s="23"/>
       <c r="H37" s="10"/>
     </row>
     <row r="38" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="13"/>
       <c r="B38" s="2"/>
-      <c r="C38" s="44"/>
-      <c r="D38" s="71"/>
-      <c r="E38" s="49"/>
-      <c r="F38" s="50"/>
+      <c r="C38" s="71"/>
+      <c r="D38" s="72"/>
+      <c r="E38" s="69"/>
+      <c r="F38" s="70"/>
       <c r="G38" s="23"/>
       <c r="H38" s="10"/>
     </row>
     <row r="39" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="13"/>
       <c r="B39" s="2"/>
-      <c r="C39" s="47"/>
-      <c r="D39" s="48"/>
-      <c r="E39" s="49"/>
-      <c r="F39" s="50"/>
+      <c r="C39" s="67"/>
+      <c r="D39" s="68"/>
+      <c r="E39" s="69"/>
+      <c r="F39" s="70"/>
       <c r="G39" s="23"/>
       <c r="H39" s="10"/>
     </row>
     <row r="40" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13"/>
       <c r="B40" s="2"/>
-      <c r="C40" s="44"/>
-      <c r="D40" s="71"/>
-      <c r="E40" s="49"/>
-      <c r="F40" s="50"/>
+      <c r="C40" s="71"/>
+      <c r="D40" s="72"/>
+      <c r="E40" s="69"/>
+      <c r="F40" s="70"/>
       <c r="G40" s="23"/>
       <c r="H40" s="10"/>
     </row>
     <row r="41" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="13"/>
       <c r="B41" s="2"/>
-      <c r="C41" s="44"/>
-      <c r="D41" s="71"/>
-      <c r="E41" s="49"/>
-      <c r="F41" s="50"/>
+      <c r="C41" s="71"/>
+      <c r="D41" s="72"/>
+      <c r="E41" s="69"/>
+      <c r="F41" s="70"/>
       <c r="G41" s="23"/>
       <c r="H41" s="10"/>
     </row>
-    <row r="42" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13"/>
       <c r="B42" s="2"/>
-      <c r="C42" s="79"/>
-      <c r="D42" s="80"/>
-      <c r="E42" s="77"/>
-      <c r="F42" s="78"/>
+      <c r="C42" s="71"/>
+      <c r="D42" s="72"/>
+      <c r="E42" s="69"/>
+      <c r="F42" s="70"/>
       <c r="G42" s="23"/>
       <c r="H42" s="10"/>
     </row>
-    <row r="43" spans="1:8" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="54" t="s">
+    <row r="43" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="13"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="71"/>
+      <c r="D43" s="72"/>
+      <c r="E43" s="69"/>
+      <c r="F43" s="70"/>
+      <c r="G43" s="23"/>
+      <c r="H43" s="10"/>
+    </row>
+    <row r="44" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="13"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="71"/>
+      <c r="D44" s="72"/>
+      <c r="E44" s="69"/>
+      <c r="F44" s="70"/>
+      <c r="G44" s="23"/>
+      <c r="H44" s="10"/>
+    </row>
+    <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="13"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="71"/>
+      <c r="D45" s="72"/>
+      <c r="E45" s="69"/>
+      <c r="F45" s="70"/>
+      <c r="G45" s="23"/>
+      <c r="H45" s="10"/>
+    </row>
+    <row r="46" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="13"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="71"/>
+      <c r="D46" s="72"/>
+      <c r="E46" s="69"/>
+      <c r="F46" s="70"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="10"/>
+    </row>
+    <row r="47" spans="1:8" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="13"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="71"/>
+      <c r="D47" s="72"/>
+      <c r="E47" s="69"/>
+      <c r="F47" s="70"/>
+      <c r="G47" s="23"/>
+    </row>
+    <row r="48" spans="1:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="B43" s="73"/>
-      <c r="C43" s="73"/>
-      <c r="D43" s="73"/>
-      <c r="E43" s="74"/>
-      <c r="F43" s="55"/>
-      <c r="G43" s="72"/>
-      <c r="H43" s="10"/>
-    </row>
-    <row r="44" spans="1:8" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="27"/>
-      <c r="B44" s="27"/>
-      <c r="C44" s="76"/>
-      <c r="D44" s="76"/>
-      <c r="E44" s="75"/>
-      <c r="F44" s="75"/>
-      <c r="G44" s="28"/>
-      <c r="H44" s="10"/>
-    </row>
-    <row r="45" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="33" t="s">
+      <c r="B48" s="58"/>
+      <c r="C48" s="58"/>
+      <c r="D48" s="58"/>
+      <c r="E48" s="59"/>
+      <c r="F48" s="60"/>
+      <c r="G48" s="61"/>
+    </row>
+    <row r="49" spans="1:7" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="79" t="s">
         <v>20</v>
       </c>
-      <c r="B45" s="34"/>
-      <c r="C45" s="82"/>
-      <c r="D45" s="83"/>
-      <c r="E45" s="83"/>
-      <c r="F45" s="83"/>
-      <c r="G45" s="84"/>
-      <c r="H45" s="10"/>
-    </row>
-    <row r="46" spans="1:8" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="52" t="s">
+      <c r="B50" s="80"/>
+      <c r="C50" s="64"/>
+      <c r="D50" s="65"/>
+      <c r="E50" s="65"/>
+      <c r="F50" s="65"/>
+      <c r="G50" s="66"/>
+    </row>
+    <row r="51" spans="1:7" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="B46" s="53"/>
-      <c r="C46" s="95"/>
-      <c r="D46" s="81"/>
-      <c r="E46" s="88" t="s">
+      <c r="B51" s="50"/>
+      <c r="C51" s="62"/>
+      <c r="D51" s="63"/>
+      <c r="E51" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="F46" s="89"/>
-      <c r="G46" s="90"/>
-      <c r="H46" s="10"/>
-    </row>
-    <row r="47" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="26" t="s">
+      <c r="F51" s="52"/>
+      <c r="G51" s="53"/>
+    </row>
+    <row r="52" spans="1:7" ht="16.5" x14ac:dyDescent="0.2">
+      <c r="A52" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B47" s="94" t="s">
+      <c r="B52" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C47" s="96"/>
-      <c r="D47" s="87"/>
-      <c r="E47" s="91" t="s">
+      <c r="C52" s="34"/>
+      <c r="D52" s="32"/>
+      <c r="E52" s="54" t="s">
         <v>18</v>
       </c>
-      <c r="F47" s="92"/>
-      <c r="G47" s="93"/>
-    </row>
-    <row r="48" spans="1:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="51" t="s">
+      <c r="F52" s="55"/>
+      <c r="G52" s="56"/>
+    </row>
+    <row r="53" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="B48" s="97"/>
-      <c r="C48" s="98"/>
-      <c r="D48" s="25"/>
-      <c r="E48" s="85" t="s">
+      <c r="B53" s="46"/>
+      <c r="C53" s="35"/>
+      <c r="D53" s="25"/>
+      <c r="E53" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="F48" s="85"/>
-      <c r="G48" s="86"/>
-    </row>
-    <row r="49" ht="42.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="50" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="51" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="F53" s="47"/>
+      <c r="G53" s="48"/>
+    </row>
   </sheetData>
-  <mergeCells count="87">
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="E48:G48"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="E46:G46"/>
-    <mergeCell ref="E47:G47"/>
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="A43:E43"/>
-    <mergeCell ref="F43:G43"/>
+  <mergeCells count="95">
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="E45:F45"/>
     <mergeCell ref="C46:D46"/>
-    <mergeCell ref="C45:G45"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="C37:D37"/>
-    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="C29:D29"/>
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="E38:F38"/>
     <mergeCell ref="E32:F32"/>
@@ -2229,54 +2259,36 @@
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="C36:D36"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="C50:G50"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="C47:D47"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="A53:B53"/>
+    <mergeCell ref="E53:G53"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="E51:G51"/>
+    <mergeCell ref="E52:G52"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="E37:F37"/>
   </mergeCells>
   <pageMargins left="0.51181102362204722" right="0.19685039370078741" top="0.31496062992125984" bottom="0" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="83" fitToHeight="0" orientation="portrait" copies="3" r:id="rId1"/>

</xml_diff>